<commit_message>
Changed EEPROM to 256kbit one for futureoroofing A/B Safe Bootloader
</commit_message>
<xml_diff>
--- a/Hardware/Controller/JLC_PCBA_BOM-DALI_EVG_Controller(V0.1).xlsx
+++ b/Hardware/Controller/JLC_PCBA_BOM-DALI_EVG_Controller(V0.1).xlsx
@@ -957,7 +957,7 @@
       <c r="C12" s="22" t="n"/>
       <c r="D12" s="22" t="inlineStr">
         <is>
-          <t>D6, D7, D8, D9</t>
+          <t>D6, D8, D9</t>
         </is>
       </c>
       <c r="E12" s="22" t="inlineStr">
@@ -966,7 +966,7 @@
         </is>
       </c>
       <c r="F12" s="30" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13">
@@ -1051,12 +1051,12 @@
     <row r="16">
       <c r="A16" s="29" t="inlineStr">
         <is>
-          <t>Header 1x9</t>
+          <t>C262302</t>
         </is>
       </c>
       <c r="B16" s="22" t="inlineStr">
         <is>
-          <t>Header 1x9</t>
+          <t>FFC/FPC Connector 10 Position 0.5mm Pitch Single-side Contact/Vertical Surface Mount</t>
         </is>
       </c>
       <c r="C16" s="22" t="n"/>
@@ -1067,7 +1067,7 @@
       </c>
       <c r="E16" s="22" t="inlineStr">
         <is>
-          <t>Header 1x9</t>
+          <t>CONN-TH-10P_AFC11-S10ICC-00</t>
         </is>
       </c>
       <c r="F16" s="30" t="n">
@@ -1524,7 +1524,7 @@
       <c r="C33" s="22" t="n"/>
       <c r="D33" s="22" t="inlineStr">
         <is>
-          <t>R27, R42</t>
+          <t>R27</t>
         </is>
       </c>
       <c r="E33" s="22" t="inlineStr">
@@ -1533,7 +1533,7 @@
         </is>
       </c>
       <c r="F33" s="30" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="34">
@@ -1773,12 +1773,12 @@
     <row r="43">
       <c r="A43" s="29" t="inlineStr">
         <is>
-          <t>M24C64-RMN6TP</t>
+          <t>AT24C256C-SSHL-T</t>
         </is>
       </c>
       <c r="B43" s="22" t="inlineStr">
         <is>
-          <t>M24C64-RMN6TP</t>
+          <t>AT24C256C-SSHL-T</t>
         </is>
       </c>
       <c r="C43" s="22" t="n"/>

</xml_diff>